<commit_message>
feat: AS IS/TO BE offices, 4-KPI bar, places balance, money mode, collapsible zones+team boxes, units; update Excel template (phase + money) and sample
</commit_message>
<xml_diff>
--- a/employee-seating-dashboard/sample-data.xlsx
+++ b/employee-seating-dashboard/sample-data.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,114 +413,138 @@
         <v>area</v>
       </c>
       <c r="D1" t="str">
-        <v>capacity</v>
+        <v>cabinet_capacity</v>
       </c>
       <c r="E1" t="str">
-        <v>cabinet_capacity</v>
+        <v>open_space_capacity</v>
       </c>
       <c r="F1" t="str">
-        <v>open_space_capacity</v>
+        <v>vip_capacity</v>
       </c>
       <c r="G1" t="str">
-        <v>vip_capacity</v>
+        <v>rent_per_sqm</v>
       </c>
       <c r="H1" t="str">
+        <v>opex_per_sqm</v>
+      </c>
+      <c r="I1" t="str">
+        <v>indexation_pct</v>
+      </c>
+      <c r="J1" t="str">
         <v>is_draft</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>comment</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="B2" t="str">
-        <v>old</v>
+        <v>asis</v>
       </c>
       <c r="C2">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="D2">
-        <v>80</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>120</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>25000</v>
+      </c>
+      <c r="H2">
+        <v>5000</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+      <c r="J2" t="str">
         <v>нет</v>
       </c>
-      <c r="I2" t="str">
-        <v>Текущая локация</v>
+      <c r="K2" t="str">
+        <v>Текущий офис</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Новый офис B</v>
+        <v>iCity 31</v>
       </c>
       <c r="B3" t="str">
-        <v>new</v>
+        <v>tobe</v>
       </c>
       <c r="C3">
-        <v>1200</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
+        <v>1768</v>
+      </c>
+      <c r="D3">
+        <v>20</v>
       </c>
       <c r="E3">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="F3">
-        <v>130</v>
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>10</v>
-      </c>
-      <c r="H3" t="str">
+        <v>32000</v>
+      </c>
+      <c r="H3">
+        <v>6000</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+      <c r="J3" t="str">
         <v>нет</v>
       </c>
-      <c r="I3" t="str">
-        <v>Основной новый офис</v>
+      <c r="K3" t="str">
+        <v>План переезда, окт 2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Новый офис C</v>
+        <v>iCity 8</v>
       </c>
       <c r="B4" t="str">
-        <v>new</v>
+        <v>tobe</v>
       </c>
       <c r="C4">
-        <v>600</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
+        <v>1500</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
       </c>
       <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4">
         <v>0</v>
       </c>
-      <c r="F4">
-        <v>60</v>
-      </c>
       <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="str">
+        <v>30000</v>
+      </c>
+      <c r="H4">
+        <v>6000</v>
+      </c>
+      <c r="I4">
+        <v>7</v>
+      </c>
+      <c r="J4" t="str">
         <v>да</v>
       </c>
-      <c r="I4" t="str">
-        <v>Черновик, уточняется</v>
+      <c r="K4" t="str">
+        <v>План, фев 2027 (черновик)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -551,22 +575,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Новый офис C</v>
+        <v>iCity 31</v>
       </c>
       <c r="B2" t="str">
-        <v>Опенспейс C</v>
+        <v>Доп. опенспейс</v>
       </c>
       <c r="C2" t="str">
         <v>open_space</v>
       </c>
       <c r="D2">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E2" t="str">
         <v>нет</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>добавочная зона</v>
       </c>
     </row>
   </sheetData>
@@ -608,7 +632,7 @@
         <v>40</v>
       </c>
       <c r="C2" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="D2" t="str">
         <v>нет</v>
@@ -628,7 +652,7 @@
         <v>25</v>
       </c>
       <c r="C3" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="D3" t="str">
         <v>нет</v>
@@ -648,7 +672,7 @@
         <v>5</v>
       </c>
       <c r="C4" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="D4" t="str">
         <v>да</v>
@@ -669,7 +693,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -705,7 +729,7 @@
         <v>Finance</v>
       </c>
       <c r="D2" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="E2" t="str">
         <v>нет</v>
@@ -728,7 +752,7 @@
         <v>Finance</v>
       </c>
       <c r="D3" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="E3" t="str">
         <v>нет</v>
@@ -745,13 +769,13 @@
         <v>Сидоров Пётр Алексеевич</v>
       </c>
       <c r="B4" t="str">
-        <v>Менеджер по продажам</v>
+        <v>Менеджер</v>
       </c>
       <c r="C4" t="str">
         <v>Sales</v>
       </c>
       <c r="D4" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="E4" t="str">
         <v>нет</v>
@@ -765,76 +789,30 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Кузнецова Мария Викторовна</v>
+        <v>Смирнов Алексей Дмитриевич</v>
       </c>
       <c r="B5" t="str">
-        <v>Менеджер по продажам</v>
+        <v>Директор</v>
       </c>
       <c r="C5" t="str">
-        <v>Sales</v>
+        <v>Руководство</v>
       </c>
       <c r="D5" t="str">
-        <v>Старый офис A</v>
+        <v>Нева 17</v>
       </c>
       <c r="E5" t="str">
-        <v>нет</v>
+        <v>да</v>
       </c>
       <c r="F5" t="str">
-        <v>удаленка</v>
+        <v>офис</v>
       </c>
       <c r="G5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Смирнов Алексей Дмитриевич</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Директор</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Руководство</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Старый офис A</v>
-      </c>
-      <c r="E6" t="str">
-        <v>да</v>
-      </c>
-      <c r="F6" t="str">
-        <v>офис</v>
-      </c>
-      <c r="G6" t="str">
         <v>Руководитель</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Николаева Ольга Павловна</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Заместитель директора</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Руководство</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Старый офис A</v>
-      </c>
-      <c r="E7" t="str">
-        <v>да</v>
-      </c>
-      <c r="F7" t="str">
-        <v>гибрид</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
style: larger fonts across cards/tabs; Excel template + sample now use Russian headers
</commit_message>
<xml_diff>
--- a/employee-seating-dashboard/sample-data.xlsx
+++ b/employee-seating-dashboard/sample-data.xlsx
@@ -404,37 +404,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>office_name</v>
+        <v>Название офиса</v>
       </c>
       <c r="B1" t="str">
-        <v>office_type</v>
+        <v>Тип офиса</v>
       </c>
       <c r="C1" t="str">
-        <v>area</v>
+        <v>Площадь</v>
       </c>
       <c r="D1" t="str">
-        <v>cabinet_capacity</v>
+        <v>Кабинеты</v>
       </c>
       <c r="E1" t="str">
-        <v>open_space_capacity</v>
+        <v>Опенспейс</v>
       </c>
       <c r="F1" t="str">
-        <v>vip_capacity</v>
+        <v>VIP-кабинеты</v>
       </c>
       <c r="G1" t="str">
-        <v>rent_per_sqm</v>
+        <v>Аренда</v>
       </c>
       <c r="H1" t="str">
-        <v>opex_per_sqm</v>
+        <v>Эксплуатация</v>
       </c>
       <c r="I1" t="str">
-        <v>indexation_pct</v>
+        <v>Индексация</v>
       </c>
       <c r="J1" t="str">
-        <v>is_draft</v>
+        <v>Черновик</v>
       </c>
       <c r="K1" t="str">
-        <v>comment</v>
+        <v>Комментарий</v>
       </c>
     </row>
     <row r="2">
@@ -442,7 +442,7 @@
         <v>Нева 17</v>
       </c>
       <c r="B2" t="str">
-        <v>asis</v>
+        <v>AS IS</v>
       </c>
       <c r="C2">
         <v>1500</v>
@@ -477,7 +477,7 @@
         <v>iCity 31</v>
       </c>
       <c r="B3" t="str">
-        <v>tobe</v>
+        <v>TO BE</v>
       </c>
       <c r="C3">
         <v>1768</v>
@@ -512,7 +512,7 @@
         <v>iCity 8</v>
       </c>
       <c r="B4" t="str">
-        <v>tobe</v>
+        <v>TO BE</v>
       </c>
       <c r="C4">
         <v>1500</v>
@@ -555,22 +555,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>office_name</v>
+        <v>Название офиса</v>
       </c>
       <c r="B1" t="str">
-        <v>zone_name</v>
+        <v>Название зоны</v>
       </c>
       <c r="C1" t="str">
-        <v>zone_type</v>
+        <v>Тип зоны</v>
       </c>
       <c r="D1" t="str">
-        <v>capacity</v>
+        <v>Вместимость</v>
       </c>
       <c r="E1" t="str">
-        <v>is_vip_zone</v>
+        <v>VIP-зона</v>
       </c>
       <c r="F1" t="str">
-        <v>comment</v>
+        <v>Комментарий</v>
       </c>
     </row>
     <row r="2">
@@ -606,22 +606,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>team_name</v>
+        <v>Название команды</v>
       </c>
       <c r="B1" t="str">
-        <v>employees_count</v>
+        <v>Количество сотрудников</v>
       </c>
       <c r="C1" t="str">
-        <v>current_office</v>
+        <v>Текущий офис</v>
       </c>
       <c r="D1" t="str">
-        <v>is_vip</v>
+        <v>VIP</v>
       </c>
       <c r="E1" t="str">
-        <v>can_split</v>
+        <v>Можно делить</v>
       </c>
       <c r="F1" t="str">
-        <v>comment</v>
+        <v>Комментарий</v>
       </c>
     </row>
     <row r="2">
@@ -697,25 +697,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>full_name</v>
+        <v>ФИО</v>
       </c>
       <c r="B1" t="str">
-        <v>position</v>
+        <v>Должность</v>
       </c>
       <c r="C1" t="str">
-        <v>team_name</v>
+        <v>Команда</v>
       </c>
       <c r="D1" t="str">
-        <v>current_office</v>
+        <v>Текущий офис</v>
       </c>
       <c r="E1" t="str">
-        <v>is_vip</v>
+        <v>VIP</v>
       </c>
       <c r="F1" t="str">
-        <v>work_format</v>
+        <v>Формат работы</v>
       </c>
       <c r="G1" t="str">
-        <v>comment</v>
+        <v>Комментарий</v>
       </c>
     </row>
     <row r="2">

</xml_diff>